<commit_message>
data: 2026-06-30 일별 수집
</commit_message>
<xml_diff>
--- a/data/daily/2026-06-30.xlsx
+++ b/data/daily/2026-06-30.xlsx
@@ -20,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -428,32 +440,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -732,7 +744,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -740,22 +752,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>오쏘몰 바이탈 m/f 14입 - 시그니처 기프트 에디션 (공식수입)</t>
+          <t>"올인원 명품비타민" 이뮨비타민 올인원 멀티비타민&amp;미네랄 프로 30병+쇼핑백증정</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>오쏘몰</t>
+          <t>닥터블릿</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>55,800원</t>
+          <t>52,900원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/8167919</t>
+          <t>https://gift.kakao.com/product/10903147</t>
         </is>
       </c>
     </row>
@@ -780,7 +792,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20,000원</t>
+          <t>24,900원</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -800,7 +812,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)+파인키위효소 1개월+저당견과류바</t>
+          <t>[그레인온] 골드 카무트 브랜드밀 효소 3개월(+선물포장)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -860,29 +872,29 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
+          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>익스트림</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>27,900원</t>
+          <t>19,900원</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7556791</t>
+          <t>https://gift.kakao.com/product/10848340</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -890,29 +902,29 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
+          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>아일로</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>58,800원</t>
+          <t>65,900원</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/12860133</t>
+          <t>https://gift.kakao.com/product/4965835</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -920,29 +932,29 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>"선물하기 1등 콜라겐" 아일로 타입1 콜라겐 비오틴 앰플 28일분 오간자 에디션+ 1입 추가 증정</t>
+          <t>[김종국 추천세트]익스트림 아르기닌정 (2개월분) &amp; 밀크씨슬 플러스 (2개월분) + 쇼핑백 증정</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>아일로</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>65,900원</t>
+          <t>27,900원</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/4965835</t>
+          <t>https://gift.kakao.com/product/7556791</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -950,29 +962,29 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[한끼통살] 닭가슴살 순삭 10팩세트(소스통살5+닭가슴살볼5)</t>
+          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>한끼통살</t>
+          <t>CJ웰케어</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>19,900원</t>
+          <t>9,900원</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/10848340</t>
+          <t>https://gift.kakao.com/product/11190137</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -980,22 +992,22 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>식물성 멜라토닌 1mg 구미 젤리 멜라메이트 1박스 (20구미) 수험생/직장인 선물</t>
+          <t>대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CJ웰케어</t>
+          <t>익스트림</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>9,900원</t>
+          <t>45,000원</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/11190137</t>
+          <t>https://gift.kakao.com/product/7417420</t>
         </is>
       </c>
     </row>
@@ -1010,22 +1022,22 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>대한민국 NO.1 김종국 트리플아르기닌 6200 (30포) + 아르기닌 추가 증정</t>
+          <t>[한끼통살] 단백질 든든형 닭가슴살 21일 식단관리+(증정)전자레인지 용기</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>익스트림</t>
+          <t>한끼통살</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>45,000원</t>
+          <t>58,800원</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://gift.kakao.com/product/7417420</t>
+          <t>https://gift.kakao.com/product/12860133</t>
         </is>
       </c>
     </row>
@@ -1073,41 +1085,41 @@
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1116,7 +1128,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -1124,29 +1136,29 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>장건강 생유산균 30캡슐 30일분</t>
+          <t>rTG오메가3 6캡슐 6일분</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>유한양행</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600651649&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000269&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1154,29 +1166,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[김우빈 PICK] 종근당건강 아임비타 비타민B 2000 30정 30일분</t>
+          <t>데일리와이즈 혈당컷 다이어트 12정 12일분</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>종근당</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591581091&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=032306201&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1184,29 +1196,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>바나바잎 10정 10일분</t>
+          <t>동국 맛있는 센시안 브이캔디 20정 20일분</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1,000원</t>
+          <t>3,000원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000278&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610910968&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>홍삼/인삼</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -1214,12 +1226,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[신혜선 PICK] 동국 마이팝 홍삼＆비타B</t>
+          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>동국제약</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1229,14 +1241,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911030&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>비타민D</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -1244,29 +1256,29 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>비타민D 4000IU 30정 30일분</t>
+          <t>[신혜선 PICK] 동국 마이팝 푸룬＆식이섬유</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>동국제약</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>2,000원</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000132&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=610911029&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>다이어트/체중관리</t>
+          <t>마그네슘</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1274,29 +1286,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[다영 PICK] 셀트리온 다이어트 한 잔 슬림 S 프레소 10포 5일분</t>
+          <t>마그네슘 샷 25ml x 5병 5일분</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=944863413&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000204&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>루테인/눈건강</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1304,7 +1316,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>rTG 오메가3 30캡슐 30일분</t>
+          <t>밀크씨슬 30정 30일분</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1319,14 +1331,14 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000145&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000134&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>마그네슘</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1334,22 +1346,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>마그네슘 30정 30일분</t>
+          <t>다이어트 홀릭 15일분</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>오브맘</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>3,000원</t>
+          <t>5,000원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000128&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=913624075&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1364,29 +1376,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>관절연골엔 MSM 60정 30일분</t>
+          <t>녹차 카테킨 6정 6일분</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>종근당건강</t>
+          <t>대웅제약</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5,000원</t>
+          <t>1,000원</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=591581121&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000282&amp;recmYn=N</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>혈행</t>
+          <t>루테인/눈건강</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1394,12 +1406,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>코엔자임 Q10 30캡슐 30일분</t>
+          <t>토비콤 루테인 지아잔틴 미니 30캡슐</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>대웅제약</t>
+          <t>안국약품</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1409,7 +1421,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=600000144&amp;recmYn=N</t>
+          <t>https://www.daisomall.co.kr/pd/pdr/SCR_PDR_0001?pdNo=611982831&amp;recmYn=N</t>
         </is>
       </c>
     </row>
@@ -1431,37 +1443,37 @@
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>순위</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>상품명</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>브랜드</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>가격</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>상품URL</t>
         </is>
@@ -1500,7 +1512,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1508,29 +1520,29 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CJ 한뿌리 흑삼지천보 진녹 30포 (1개월분) (온)</t>
+          <t>[10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>한뿌리</t>
+          <t>라이필</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>250,000원</t>
+          <t>15,840원</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247763&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=2</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>멀티비타민/종합비타민</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1538,22 +1550,22 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[10일콜라겐/모공,목주름/PDRN] 라이필 더마콜라겐 시그니처RN (10일분)</t>
+          <t>오쏘몰 이뮨 멀티비타민&amp;미네랄 14입 단품/기획</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>라이필</t>
+          <t>오쏘몰</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>15,840원</t>
+          <t>55,900원</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000259411&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000193086&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=3</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1632,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>프로바이오틱스/유산균</t>
+          <t>다이어트/체중관리</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -1628,29 +1640,29 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
+          <t>[7월 올영픽/서현PICK] 콜레올로지 PRO 600mg*30(+10)/60정 단품</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>덴프스</t>
+          <t>푸드올로지</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>30,400원</t>
+          <t>22,900원</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000206861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000175634&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=6</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>피부/미용</t>
+          <t>기타/특수목적</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -1658,29 +1670,29 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>[6월 올영픽/윤광UP]온리추얼 글로우업 글루타치온 콜라겐 7포 (+1포 증정)</t>
+          <t>[6월 올영픽/곽민경 PICK] 생활약속 기분전환 알파플러스 10포 (+1포 증정기획)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>온리추얼</t>
+          <t>생활약속</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15,900원</t>
+          <t>15,400원</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000247570&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000180121&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=7</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -1688,29 +1700,29 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>[6월 올영픽] 온리추얼 리셋 브이라인 7포 (+1포 증정) (8일분)</t>
+          <t>[포켓몬 에디션] 덴마크 유산균이야기 30캡슐 1+1 (+꼬부기 러기지택) (60일분)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>온리추얼</t>
+          <t>덴프스</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>14,900원</t>
+          <t>30,400원</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000249190&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=8</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000206861&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>프로바이오틱스/유산균</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1718,29 +1730,29 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[7월 올영픽] 오니스트 케라그로우 망고 14일 루틴 단품/기획(+2포)</t>
+          <t>[덴프스] 덴마크 유산균이야기 우먼 2개월분(질유산균) + 철분 헤모케어 3포 증정</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>오니스트</t>
+          <t>덴프스</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>28,900원</t>
+          <t>37,050원</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000241378&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000202658&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=9</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>기타/특수목적</t>
+          <t>피부/미용</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -1748,22 +1760,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>[7월 올영픽] 식물성 멜라토닌 함유 멜라메이트 구미/로우슈가/버라이어티 구미 20/40/50구미</t>
+          <t>솔가 비오틴 5000 (100캡슐/100일분)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>멜라메이트</t>
+          <t>솔가</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13,000원</t>
+          <t>50,000원</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000223554&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
+          <t>https://www.oliveyoung.co.kr/store/goods/getGoodsDetail.do?goodsNo=A000000138890&amp;dispCatNo=90000010009&amp;trackingCd=Best_Sellingbest&amp;t_page=랭킹&amp;t_click=판매랭킹_건강식품_상품상세&amp;t_number=10</t>
         </is>
       </c>
     </row>
@@ -1790,32 +1802,32 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>카테고리</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>전체</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>비율(%)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>카카오선물하기</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>다이소몰</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>올리브영</t>
         </is>
@@ -1828,19 +1840,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -1872,16 +1884,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -1916,16 +1928,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -1938,16 +1950,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -1960,16 +1972,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -1982,19 +1994,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C9" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D9" t="n">
         <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -2013,10 +2025,10 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -2048,19 +2060,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C12" t="n">
-        <v>27.5</v>
+        <v>22.5</v>
       </c>
       <c r="D12" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>2</v>
-      </c>
-      <c r="F12" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="13">

</xml_diff>